<commit_message>
fix(demo-data): align weekly budget dates with the demo calendar
The business-unit weekly budget sheet used week dates (07-08, 07-15,
07-22) that did not match the calendar week starts (07-06, 07-13,
07-20), so the weekly calculation never found a budget and all target
and final amounts stayed empty. Align the dates; amounts are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo-data/基本数据模板_第十三版_通用供应链演示版.xlsx
+++ b/demo-data/基本数据模板_第十三版_通用供应链演示版.xlsx
@@ -7178,7 +7178,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -7215,7 +7215,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -7252,7 +7252,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">

</xml_diff>